<commit_message>
feat(F-NAR-019): TREE-COL-005 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-005.xlsx
+++ b/stories/arbres/TREE-COL-005.xlsx
@@ -7092,7 +7092,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>s'il te plaît | s'il te plait | sil te plait | please</t>
+          <t>s'il te plaît | s'il te plait | sil te plait</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -15006,17 +15006,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Le pain de la phrase entière chauffe le tissu. L'auvent n'a pas touché la croûte. Elle a eu toute la phrase. Oui. Merci, le col était ouvert. Le manteau s'ouvre, une bouffée d'air de soupe. Le livre sous le bras est resté à l'école. Un tic de gouttière, puis le silence du pain.</t>
+          <t>Le pain de la phrase entière chauffe le tissu. L'auvent n'a pas touché la croûte. Elle a eu toute la phrase. Toute la phrase, oui. Merci, le col était ouvert. Le manteau s'ouvre, une bouffée d'air de soupe. Le livre sous le bras est resté à l'école. Un tic de gouttière, puis le silence du pain.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le pain de la phrase entière chauffe le tissu. L'auvent n'a pas touché la croûte. Elle a eu toute la phrase. Oui. Merci, le col était ouvert. Le manteau s'ouvre, une bouffée d'air de soupe. Le livre sous le bras est resté à l'école. Un tic de gouttière, puis le silence du pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le pain de la phrase entière chauffe le tissu. L'auvent n'a pas touché la croûte. Elle a eu toute la phrase. Toute la phrase, oui. Merci, le col était ouvert. Le manteau s'ouvre, une bouffée d'air de soupe. Le livre sous le bras est resté à l'école. Un tic de gouttière, puis le silence du pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le pain de la phrase entière chauffe le tissu. L'auvent n'a pas touché la croûte. Elle a eu toute la phrase. Oui. Merci, le col était ouvert. Le manteau s'ouvre, une bouffée d'air de soupe. Le livre sous le bras est resté à l'école. Un tic de gouttière, puis le silence du pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le pain de la phrase entière chauffe le tissu. L'auvent n'a pas touché la croûte. Elle a eu toute la phrase. Toute la phrase, oui. Merci, le col était ouvert. Le manteau s'ouvre, une bouffée d'air de soupe. Le livre sous le bras est resté à l'école. Un tic de gouttière, puis le silence du pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15157,7 +15157,7 @@
           <t>narrateur|Le pain de la phrase entière chauffe le tissu.
 narrateur|L'auvent n'a pas touché la croûte.
 enfant-m|Elle a eu toute la phrase.
-maitresse|Oui.
+maman|Toute la phrase, oui.
 papa|Merci, le col était ouvert.
 narrateur|Le manteau s'ouvre, une bouffée d'air de soupe.
 narrateur|Le livre sous le bras est resté à l'école.
@@ -17447,7 +17447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17504,6 +17504,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>